<commit_message>
Prefiltro, validación (248 OK) y lista para Investigación con hoja de preguntas de prueba
</commit_message>
<xml_diff>
--- a/corpus/md/reporte_validacion.xlsx
+++ b/corpus/md/reporte_validacion.xlsx
@@ -421,7 +421,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Archivos por estado y colección (validación del 2026-10-15 02:01)</t>
+          <t>Archivos por estado y colección (validación del 2026-10-15 02:22)</t>
         </is>
       </c>
     </row>
@@ -459,7 +459,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -468,7 +468,7 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -478,16 +478,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C4" t="n">
         <v>76</v>
       </c>
       <c r="D4" t="n">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="E4" t="n">
-        <v>240</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5">
@@ -560,10 +560,10 @@
         <v>79</v>
       </c>
       <c r="D8" t="n">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="E8" t="n">
-        <v>257</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q258"/>
+  <dimension ref="A1:Q276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3655,10 +3655,14 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q50" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3716,10 +3720,14 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3777,10 +3785,14 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q52" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3899,10 +3911,14 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4021,10 +4037,14 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q56" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4082,10 +4102,14 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4147,10 +4171,14 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q58" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4208,10 +4236,14 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q59" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4269,10 +4301,14 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q60" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4330,10 +4366,14 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q61" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -16019,7 +16059,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -16029,7 +16069,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>d) PDF directo</t>
+          <t>e) PDF local</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -16039,23 +16079,23 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>683</t>
+          <t>9013</t>
         </is>
       </c>
       <c r="F251" t="n">
-        <v>623</v>
+        <v>8977</v>
       </c>
       <c r="G251" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H251" t="n">
-        <v>1365</v>
+        <v>31194</v>
       </c>
       <c r="I251" t="n">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="J251" t="n">
-        <v>0.36</v>
+        <v>0.2</v>
       </c>
       <c r="K251" t="inlineStr"/>
       <c r="L251" t="b">
@@ -16066,12 +16106,12 @@
       </c>
       <c r="N251" t="inlineStr">
         <is>
-          <t>Kits aprobados por el Servicio, segun instructivo tecnico pertinente (D-ATR-AAT-096, version 01)</t>
+          <t>Codes and Manuals: Terrestrial Manual, Capitulo 1.1.2 Collection, submission and storage of diagnostic specimens</t>
         </is>
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>corpus\md\diagnostico\D11.md</t>
+          <t>corpus\md\diagnostico\D10.md</t>
         </is>
       </c>
       <c r="P251" t="inlineStr">
@@ -16079,12 +16119,16 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="Q251" t="inlineStr"/>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>título 74/100, aceptado por tener 8977 palabras (&gt; 1500)</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -16104,23 +16148,23 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>8630</t>
+          <t>683</t>
         </is>
       </c>
       <c r="F252" t="n">
-        <v>8247</v>
+        <v>623</v>
       </c>
       <c r="G252" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="H252" t="n">
-        <v>3892</v>
+        <v>1365</v>
       </c>
       <c r="I252" t="n">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="J252" t="n">
-        <v>0.21</v>
+        <v>0.36</v>
       </c>
       <c r="K252" t="inlineStr"/>
       <c r="L252" t="b">
@@ -16131,12 +16175,12 @@
       </c>
       <c r="N252" t="inlineStr">
         <is>
-          <t>Manual Terrestre de la OMSA, Capitulo 2.2.1: Desarrollo y optimizacion de los ensayos de deteccion de anticuerpos</t>
+          <t>Kits aprobados por el Servicio, segun instructivo tecnico pertinente (D-ATR-AAT-096, version 01)</t>
         </is>
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>corpus\md\diagnostico\D19.md</t>
+          <t>corpus\md\diagnostico\D11.md</t>
         </is>
       </c>
       <c r="P252" t="inlineStr">
@@ -16144,16 +16188,12 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="Q252" t="inlineStr">
-        <is>
-          <t>título 51/100, aceptado por tener 8247 palabras (&gt; 1500)</t>
-        </is>
-      </c>
+      <c r="Q252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -16163,29 +16203,33 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>c) Web</t>
+          <t>e) PDF local</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>aviar</t>
+          <t>porcino</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>173</t>
         </is>
       </c>
       <c r="F253" t="n">
-        <v>200</v>
-      </c>
-      <c r="G253" t="inlineStr"/>
-      <c r="H253" t="inlineStr"/>
+        <v>173</v>
+      </c>
+      <c r="G253" t="n">
+        <v>1</v>
+      </c>
+      <c r="H253" t="n">
+        <v>1108</v>
+      </c>
       <c r="I253" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="J253" t="n">
-        <v>0.59</v>
+        <v>0</v>
       </c>
       <c r="K253" t="inlineStr"/>
       <c r="L253" t="b">
@@ -16196,12 +16240,12 @@
       </c>
       <c r="N253" t="inlineStr">
         <is>
-          <t>IDEXX AI MultiS-Screen Ab Test - pagina de producto</t>
+          <t>IDEXX PRRS X3 Ab Test - pagina de producto</t>
         </is>
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>corpus\md\diagnostico\D20.md</t>
+          <t>corpus\md\diagnostico\D13.md</t>
         </is>
       </c>
       <c r="P253" t="inlineStr">
@@ -16211,14 +16255,14 @@
       </c>
       <c r="Q253" t="inlineStr">
         <is>
-          <t>título 76/100 (&lt; 80) y 200 palabras</t>
+          <t>título 64/100 (&lt; 80) y 173 palabras</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -16228,49 +16272,49 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>d) PDF directo</t>
+          <t>e) PDF local</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>aviar</t>
+          <t>porcino</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>7931</t>
+          <t>299</t>
         </is>
       </c>
       <c r="F254" t="n">
-        <v>7675</v>
+        <v>299</v>
       </c>
       <c r="G254" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="H254" t="n">
-        <v>2712</v>
+        <v>1754</v>
       </c>
       <c r="I254" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="J254" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="K254" t="inlineStr"/>
       <c r="L254" t="b">
         <v>0</v>
       </c>
       <c r="M254" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N254" t="inlineStr">
         <is>
-          <t>Instructivo Tecnico para el Diagnostico de Influenza Aviar mediante ELISA y RT-PCR en tiempo real (D-ATR-AAT-013, version 03)</t>
+          <t>Best practices for using the IDEXX PRRS Oral Fluids Ab Test</t>
         </is>
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>corpus\md\diagnostico\D22.md</t>
+          <t>corpus\md\diagnostico\D14.md</t>
         </is>
       </c>
       <c r="P254" t="inlineStr">
@@ -16283,7 +16327,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>D23</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -16293,45 +16337,49 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>a) Europe PMC</t>
+          <t>e) PDF local</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>aviar</t>
+          <t>porcino</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>10036</t>
+          <t>243</t>
         </is>
       </c>
       <c r="F255" t="n">
-        <v>10034</v>
-      </c>
-      <c r="G255" t="inlineStr"/>
-      <c r="H255" t="inlineStr"/>
+        <v>243</v>
+      </c>
+      <c r="G255" t="n">
+        <v>1</v>
+      </c>
+      <c r="H255" t="n">
+        <v>1755</v>
+      </c>
       <c r="I255" t="n">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="J255" t="n">
-        <v>0.09</v>
+        <v>0.25</v>
       </c>
       <c r="K255" t="inlineStr"/>
       <c r="L255" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M255" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N255" t="inlineStr">
         <is>
-          <t>Comparison of whole blood on filter strips with serum for avian influenza virus antibody detection in wild birds</t>
+          <t>IDEXX PRRS Oral Fluids Ab Test (North America) - pagina de producto</t>
         </is>
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>corpus\md\diagnostico\D23.md</t>
+          <t>corpus\md\diagnostico\D15.md</t>
         </is>
       </c>
       <c r="P255" t="inlineStr">
@@ -16344,7 +16392,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>D27</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -16354,49 +16402,49 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>d) PDF directo</t>
+          <t>e) PDF local</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>aviar</t>
+          <t>porcino</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2985</t>
+          <t>12943</t>
         </is>
       </c>
       <c r="F256" t="n">
-        <v>2882</v>
+        <v>10743</v>
       </c>
       <c r="G256" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="H256" t="n">
-        <v>2436</v>
+        <v>3283</v>
       </c>
       <c r="I256" t="n">
-        <v>90</v>
+        <v>57</v>
       </c>
       <c r="J256" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="K256" t="inlineStr"/>
       <c r="L256" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M256" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N256" t="inlineStr">
         <is>
-          <t>Avian Sample Collection for Influenza A and Newcastle Disease (NVSL-WI-0023)</t>
+          <t>Manual Terrestre de la OMSA, Capitulo 3.9.6: Sindrome reproductivo y respiratorio porcino (PRRS)</t>
         </is>
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>corpus\md\diagnostico\D27.md</t>
+          <t>corpus\md\diagnostico\D16.md</t>
         </is>
       </c>
       <c r="P256" t="inlineStr">
@@ -16404,12 +16452,16 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="Q256" t="inlineStr"/>
+      <c r="Q256" t="inlineStr">
+        <is>
+          <t>título 57/100, aceptado por tener 10743 palabras (&gt; 1500)</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D17</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -16419,49 +16471,49 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>d) PDF directo</t>
+          <t>e) PDF local</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>porcino</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>17666</t>
+          <t>3066</t>
         </is>
       </c>
       <c r="F257" t="n">
-        <v>17213</v>
+        <v>2864</v>
       </c>
       <c r="G257" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="H257" t="n">
-        <v>4374</v>
+        <v>4520</v>
       </c>
       <c r="I257" t="n">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="J257" t="n">
-        <v>0.17</v>
+        <v>0.11</v>
       </c>
       <c r="K257" t="inlineStr"/>
       <c r="L257" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M257" t="b">
         <v>0</v>
       </c>
       <c r="N257" t="inlineStr">
         <is>
-          <t>Manual Terrestre de la OMSA, Capitulo 1.1.6: Validacion de las pruebas de diagnostico de las enfermedades infecciosas de animales terrestres</t>
+          <t>Field application of a commercial PRRSV oral fluid antibody ELISA</t>
         </is>
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>corpus\md\diagnostico\D7.md</t>
+          <t>corpus\md\diagnostico\D17.md</t>
         </is>
       </c>
       <c r="P257" t="inlineStr">
@@ -16471,14 +16523,14 @@
       </c>
       <c r="Q257" t="inlineStr">
         <is>
-          <t>título 57/100, aceptado por tener 17213 palabras (&gt; 1500)</t>
+          <t>título 76/100, aceptado por tener 2864 palabras (&gt; 1500)</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -16488,33 +16540,33 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>d) PDF directo</t>
+          <t>e) PDF local</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>aviar</t>
+          <t>porcino</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>18264</t>
+          <t>6480</t>
         </is>
       </c>
       <c r="F258" t="n">
-        <v>14902</v>
+        <v>5478</v>
       </c>
       <c r="G258" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="H258" t="n">
-        <v>3523</v>
+        <v>3403</v>
       </c>
       <c r="I258" t="n">
-        <v>52</v>
+        <v>90</v>
       </c>
       <c r="J258" t="n">
-        <v>0.2</v>
+        <v>0.33</v>
       </c>
       <c r="K258" t="inlineStr"/>
       <c r="L258" t="b">
@@ -16525,24 +16577,1206 @@
       </c>
       <c r="N258" t="inlineStr">
         <is>
+          <t>Kinetics of the PRRSV humoral immune response in swine serum and oral fluids collected from individual boars</t>
+        </is>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D18.md</t>
+        </is>
+      </c>
+      <c r="P258" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>D19</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>d) PDF directo</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>8630</t>
+        </is>
+      </c>
+      <c r="F259" t="n">
+        <v>8247</v>
+      </c>
+      <c r="G259" t="n">
+        <v>14</v>
+      </c>
+      <c r="H259" t="n">
+        <v>3892</v>
+      </c>
+      <c r="I259" t="n">
+        <v>51</v>
+      </c>
+      <c r="J259" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="K259" t="inlineStr"/>
+      <c r="L259" t="b">
+        <v>0</v>
+      </c>
+      <c r="M259" t="b">
+        <v>0</v>
+      </c>
+      <c r="N259" t="inlineStr">
+        <is>
+          <t>Manual Terrestre de la OMSA, Capitulo 2.2.1: Desarrollo y optimizacion de los ensayos de deteccion de anticuerpos</t>
+        </is>
+      </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D19.md</t>
+        </is>
+      </c>
+      <c r="P259" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q259" t="inlineStr">
+        <is>
+          <t>título 51/100, aceptado por tener 8247 palabras (&gt; 1500)</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>aviar</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="F260" t="n">
+        <v>187</v>
+      </c>
+      <c r="G260" t="n">
+        <v>1</v>
+      </c>
+      <c r="H260" t="n">
+        <v>1276</v>
+      </c>
+      <c r="I260" t="n">
+        <v>81</v>
+      </c>
+      <c r="J260" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="K260" t="inlineStr"/>
+      <c r="L260" t="b">
+        <v>0</v>
+      </c>
+      <c r="M260" t="b">
+        <v>0</v>
+      </c>
+      <c r="N260" t="inlineStr">
+        <is>
+          <t>IDEXX AI MultiS-Screen Ab Test - pagina de producto</t>
+        </is>
+      </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D20.md</t>
+        </is>
+      </c>
+      <c r="P260" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>D21</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>aviar</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>6296</t>
+        </is>
+      </c>
+      <c r="F261" t="n">
+        <v>6024</v>
+      </c>
+      <c r="G261" t="n">
+        <v>18</v>
+      </c>
+      <c r="H261" t="n">
+        <v>2497</v>
+      </c>
+      <c r="I261" t="n">
+        <v>80</v>
+      </c>
+      <c r="J261" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K261" t="inlineStr"/>
+      <c r="L261" t="b">
+        <v>1</v>
+      </c>
+      <c r="M261" t="b">
+        <v>1</v>
+      </c>
+      <c r="N261" t="inlineStr">
+        <is>
+          <t>Limited detection of antibodies to clade 2.3.4.4 A/goose/Guangdong/1/1996 lineage HPAI virus in North American waterfowl</t>
+        </is>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D21.md</t>
+        </is>
+      </c>
+      <c r="P261" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>D22</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>d) PDF directo</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>aviar</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>7931</t>
+        </is>
+      </c>
+      <c r="F262" t="n">
+        <v>7675</v>
+      </c>
+      <c r="G262" t="n">
+        <v>20</v>
+      </c>
+      <c r="H262" t="n">
+        <v>2712</v>
+      </c>
+      <c r="I262" t="n">
+        <v>90</v>
+      </c>
+      <c r="J262" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K262" t="inlineStr"/>
+      <c r="L262" t="b">
+        <v>0</v>
+      </c>
+      <c r="M262" t="b">
+        <v>1</v>
+      </c>
+      <c r="N262" t="inlineStr">
+        <is>
+          <t>Instructivo Tecnico para el Diagnostico de Influenza Aviar mediante ELISA y RT-PCR en tiempo real (D-ATR-AAT-013, version 03)</t>
+        </is>
+      </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D22.md</t>
+        </is>
+      </c>
+      <c r="P262" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>a) Europe PMC</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>aviar</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>10036</t>
+        </is>
+      </c>
+      <c r="F263" t="n">
+        <v>10034</v>
+      </c>
+      <c r="G263" t="inlineStr"/>
+      <c r="H263" t="inlineStr"/>
+      <c r="I263" t="n">
+        <v>100</v>
+      </c>
+      <c r="J263" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="K263" t="inlineStr"/>
+      <c r="L263" t="b">
+        <v>1</v>
+      </c>
+      <c r="M263" t="b">
+        <v>1</v>
+      </c>
+      <c r="N263" t="inlineStr">
+        <is>
+          <t>Comparison of whole blood on filter strips with serum for avian influenza virus antibody detection in wild birds</t>
+        </is>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D23.md</t>
+        </is>
+      </c>
+      <c r="P263" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>D24</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>aviar</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>10498</t>
+        </is>
+      </c>
+      <c r="F264" t="n">
+        <v>10345</v>
+      </c>
+      <c r="G264" t="n">
+        <v>13</v>
+      </c>
+      <c r="H264" t="n">
+        <v>5481</v>
+      </c>
+      <c r="I264" t="n">
+        <v>100</v>
+      </c>
+      <c r="J264" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K264" t="inlineStr"/>
+      <c r="L264" t="b">
+        <v>1</v>
+      </c>
+      <c r="M264" t="b">
+        <v>1</v>
+      </c>
+      <c r="N264" t="inlineStr">
+        <is>
+          <t>Surveillance of live birds for active and past infections reveals the impact of highly pathogenic H5N1 on seabird populations in Atlantic Canada</t>
+        </is>
+      </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D24.md</t>
+        </is>
+      </c>
+      <c r="P264" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>porcino</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>2719</t>
+        </is>
+      </c>
+      <c r="F265" t="n">
+        <v>2719</v>
+      </c>
+      <c r="G265" t="n">
+        <v>4</v>
+      </c>
+      <c r="H265" t="n">
+        <v>4652</v>
+      </c>
+      <c r="I265" t="n">
+        <v>81</v>
+      </c>
+      <c r="J265" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="K265" t="inlineStr"/>
+      <c r="L265" t="b">
+        <v>0</v>
+      </c>
+      <c r="M265" t="b">
+        <v>1</v>
+      </c>
+      <c r="N265" t="inlineStr">
+        <is>
+          <t>Evaluation of three commercially available influenza A type specific blocking ELISAs for seroepidemiological studies of influenza A virus infection in pigs</t>
+        </is>
+      </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D25.md</t>
+        </is>
+      </c>
+      <c r="P265" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>D27</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>d) PDF directo</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>aviar</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>2985</t>
+        </is>
+      </c>
+      <c r="F266" t="n">
+        <v>2882</v>
+      </c>
+      <c r="G266" t="n">
+        <v>8</v>
+      </c>
+      <c r="H266" t="n">
+        <v>2436</v>
+      </c>
+      <c r="I266" t="n">
+        <v>90</v>
+      </c>
+      <c r="J266" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K266" t="inlineStr"/>
+      <c r="L266" t="b">
+        <v>0</v>
+      </c>
+      <c r="M266" t="b">
+        <v>0</v>
+      </c>
+      <c r="N266" t="inlineStr">
+        <is>
+          <t>Avian Sample Collection for Influenza A and Newcastle Disease (NVSL-WI-0023)</t>
+        </is>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D27.md</t>
+        </is>
+      </c>
+      <c r="P266" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>aviar</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>21855</t>
+        </is>
+      </c>
+      <c r="F267" t="n">
+        <v>20976</v>
+      </c>
+      <c r="G267" t="n">
+        <v>57</v>
+      </c>
+      <c r="H267" t="n">
+        <v>2501</v>
+      </c>
+      <c r="I267" t="n">
+        <v>83</v>
+      </c>
+      <c r="J267" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="K267" t="inlineStr"/>
+      <c r="L267" t="b">
+        <v>0</v>
+      </c>
+      <c r="M267" t="b">
+        <v>1</v>
+      </c>
+      <c r="N267" t="inlineStr">
+        <is>
+          <t>Plan de Contingencia Influenza Aviar (IA), Version 6.0</t>
+        </is>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D3.md</t>
+        </is>
+      </c>
+      <c r="P267" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>D32</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>12959</t>
+        </is>
+      </c>
+      <c r="F268" t="n">
+        <v>11622</v>
+      </c>
+      <c r="G268" t="n">
+        <v>18</v>
+      </c>
+      <c r="H268" t="n">
+        <v>4646</v>
+      </c>
+      <c r="I268" t="n">
+        <v>100</v>
+      </c>
+      <c r="J268" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="K268" t="inlineStr"/>
+      <c r="L268" t="b">
+        <v>1</v>
+      </c>
+      <c r="M268" t="b">
+        <v>0</v>
+      </c>
+      <c r="N268" t="inlineStr">
+        <is>
+          <t>MIQE 2.0: Revision of the Minimum Information for Publication of Quantitative Real-Time PCR Experiments Guidelines</t>
+        </is>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D32.md</t>
+        </is>
+      </c>
+      <c r="P268" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q268" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>D33</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>aviar</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>4945</t>
+        </is>
+      </c>
+      <c r="F269" t="n">
+        <v>4943</v>
+      </c>
+      <c r="G269" t="n">
+        <v>5</v>
+      </c>
+      <c r="H269" t="n">
+        <v>6556</v>
+      </c>
+      <c r="I269" t="n">
+        <v>100</v>
+      </c>
+      <c r="J269" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="K269" t="inlineStr"/>
+      <c r="L269" t="b">
+        <v>0</v>
+      </c>
+      <c r="M269" t="b">
+        <v>1</v>
+      </c>
+      <c r="N269" t="inlineStr">
+        <is>
+          <t>Development of a real-time reverse transcriptase PCR assay for type A influenza virus and the avian H5 and H7 hemagglutinin subtypes</t>
+        </is>
+      </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D33.md</t>
+        </is>
+      </c>
+      <c r="P269" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>D34</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>porcino</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>9021</t>
+        </is>
+      </c>
+      <c r="F270" t="n">
+        <v>8889</v>
+      </c>
+      <c r="G270" t="n">
+        <v>12</v>
+      </c>
+      <c r="H270" t="n">
+        <v>4976</v>
+      </c>
+      <c r="I270" t="n">
+        <v>100</v>
+      </c>
+      <c r="J270" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="K270" t="inlineStr"/>
+      <c r="L270" t="b">
+        <v>1</v>
+      </c>
+      <c r="M270" t="b">
+        <v>0</v>
+      </c>
+      <c r="N270" t="inlineStr">
+        <is>
+          <t>Guidelines for oral fluid-based surveillance of viral pathogens in swine</t>
+        </is>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D34.md</t>
+        </is>
+      </c>
+      <c r="P270" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q270" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>D35</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>porcino</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>7078</t>
+        </is>
+      </c>
+      <c r="F271" t="n">
+        <v>4080</v>
+      </c>
+      <c r="G271" t="n">
+        <v>8</v>
+      </c>
+      <c r="H271" t="n">
+        <v>3784</v>
+      </c>
+      <c r="I271" t="n">
+        <v>100</v>
+      </c>
+      <c r="J271" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="K271" t="inlineStr"/>
+      <c r="L271" t="b">
+        <v>1</v>
+      </c>
+      <c r="M271" t="b">
+        <v>0</v>
+      </c>
+      <c r="N271" t="inlineStr">
+        <is>
+          <t>The use of oral fluid diagnostics in swine medicine</t>
+        </is>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D35.md</t>
+        </is>
+      </c>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>21892</t>
+        </is>
+      </c>
+      <c r="F272" t="n">
+        <v>21809</v>
+      </c>
+      <c r="G272" t="n">
+        <v>60</v>
+      </c>
+      <c r="H272" t="n">
+        <v>2692</v>
+      </c>
+      <c r="I272" t="n">
+        <v>97</v>
+      </c>
+      <c r="J272" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>comprar</t>
+        </is>
+      </c>
+      <c r="L272" t="b">
+        <v>0</v>
+      </c>
+      <c r="M272" t="b">
+        <v>0</v>
+      </c>
+      <c r="N272" t="inlineStr">
+        <is>
+          <t>Guia sobre la reglamentacion relativa al transporte de sustancias infecciosas 2019-2020</t>
+        </is>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D5.md</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>4602</t>
+        </is>
+      </c>
+      <c r="F273" t="n">
+        <v>4147</v>
+      </c>
+      <c r="G273" t="n">
+        <v>9</v>
+      </c>
+      <c r="H273" t="n">
+        <v>3307</v>
+      </c>
+      <c r="I273" t="n">
+        <v>53</v>
+      </c>
+      <c r="J273" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="K273" t="inlineStr"/>
+      <c r="L273" t="b">
+        <v>1</v>
+      </c>
+      <c r="M273" t="b">
+        <v>0</v>
+      </c>
+      <c r="N273" t="inlineStr">
+        <is>
+          <t>Manual Terrestre de la OMSA, Capitulo 1.1.5: Gestion de calidad en los laboratorios de pruebas veterinarias</t>
+        </is>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D6.md</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>título 53/100, aceptado por tener 4147 palabras (&gt; 1500)</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>d) PDF directo</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>17666</t>
+        </is>
+      </c>
+      <c r="F274" t="n">
+        <v>17213</v>
+      </c>
+      <c r="G274" t="n">
+        <v>27</v>
+      </c>
+      <c r="H274" t="n">
+        <v>4374</v>
+      </c>
+      <c r="I274" t="n">
+        <v>57</v>
+      </c>
+      <c r="J274" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="K274" t="inlineStr"/>
+      <c r="L274" t="b">
+        <v>0</v>
+      </c>
+      <c r="M274" t="b">
+        <v>0</v>
+      </c>
+      <c r="N274" t="inlineStr">
+        <is>
+          <t>Manual Terrestre de la OMSA, Capitulo 1.1.6: Validacion de las pruebas de diagnostico de las enfermedades infecciosas de animales terrestres</t>
+        </is>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D7.md</t>
+        </is>
+      </c>
+      <c r="P274" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>título 57/100, aceptado por tener 17213 palabras (&gt; 1500)</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>d) PDF directo</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>aviar</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>18264</t>
+        </is>
+      </c>
+      <c r="F275" t="n">
+        <v>14902</v>
+      </c>
+      <c r="G275" t="n">
+        <v>28</v>
+      </c>
+      <c r="H275" t="n">
+        <v>3523</v>
+      </c>
+      <c r="I275" t="n">
+        <v>52</v>
+      </c>
+      <c r="J275" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K275" t="inlineStr"/>
+      <c r="L275" t="b">
+        <v>1</v>
+      </c>
+      <c r="M275" t="b">
+        <v>1</v>
+      </c>
+      <c r="N275" t="inlineStr">
+        <is>
           <t>Manual Terrestre de la OMSA, Capitulo 3.3.4: Influenza aviar (incluida la infeccion por los virus de la influenza aviar altamente patogenos)</t>
         </is>
       </c>
-      <c r="O258" t="inlineStr">
+      <c r="O275" t="inlineStr">
         <is>
           <t>corpus\md\diagnostico\D8.md</t>
         </is>
       </c>
-      <c r="P258" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q258" t="inlineStr">
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q275" t="inlineStr">
         <is>
           <t>título 52/100, aceptado por tener 14902 palabras (&gt; 1500)</t>
         </is>
       </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>diagnostico</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>e) PDF local</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>9278</t>
+        </is>
+      </c>
+      <c r="F276" t="n">
+        <v>9254</v>
+      </c>
+      <c r="G276" t="n">
+        <v>32</v>
+      </c>
+      <c r="H276" t="n">
+        <v>2245</v>
+      </c>
+      <c r="I276" t="n">
+        <v>98</v>
+      </c>
+      <c r="J276" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="K276" t="inlineStr"/>
+      <c r="L276" t="b">
+        <v>0</v>
+      </c>
+      <c r="M276" t="b">
+        <v>0</v>
+      </c>
+      <c r="N276" t="inlineStr">
+        <is>
+          <t>IDEXX Reference Laboratories: Specimen Collection Guidelines</t>
+        </is>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>corpus\md\diagnostico\D9.md</t>
+        </is>
+      </c>
+      <c r="P276" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q276" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16555,7 +17789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16643,10 +17877,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>PALABRAS_PAGO</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>FRASES_PAGO</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Purchase access, Access through your institution, Log in, Subscribe, Comprar</t>
         </is>

</xml_diff>

<commit_message>
Excluye BIO-123, BIO-126 y BIO-138 (IA, no base veterinaria) y marca 'retrieval-augmented' y 'multi-agent'
</commit_message>
<xml_diff>
--- a/corpus/md/reporte_validacion.xlsx
+++ b/corpus/md/reporte_validacion.xlsx
@@ -415,13 +415,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Archivos por estado y colección (validación del 2026-10-15 02:55)</t>
+          <t>Archivos por estado y colección (validación del 2026-10-15 03:18)</t>
         </is>
       </c>
     </row>
@@ -455,95 +455,114 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Excluido</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>75</v>
+        <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>248</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Página equivocada</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>72</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>76</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Revisar título</t>
+          <t>Página equivocada</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Solo resumen</t>
+          <t>Revisar título</t>
         </is>
       </c>
       <c r="B6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C6" t="n">
         <v>0</v>
       </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Solo resumen</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B8" t="n">
         <v>87</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C8" t="n">
         <v>79</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D8" t="n">
         <v>98</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E8" t="n">
         <v>264</v>
       </c>
     </row>
@@ -3636,10 +3655,14 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q50" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3697,10 +3720,14 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3758,10 +3785,14 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="Q52" t="inlineStr"/>
+          <t>Excluido</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>el prefiltro la sacó (excluida a mano o duplicada)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">

</xml_diff>